<commit_message>
Snowflake COP-SF-05 breakdown rev 1: area amounts per Ruslan markup
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WgFPTBsAevVc5EmsheUHsa
</commit_message>
<xml_diff>
--- a/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
+++ b/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
@@ -459,7 +459,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>COP-SF-05 Bulletin 3 Revision - Snowflake Fitout, 7 Times Square Fl 29-31 - Northern Wolves AC - 09/29/2026</t>
+          <t>COP-SF-05 Bulletin 3 Revision - Snowflake Fitout, 7 Times Square Fl 29-31 - Northern Wolves AC - 09/30/2026</t>
         </is>
       </c>
     </row>
@@ -545,14 +545,14 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E4" s="2">
         <f>D4*125</f>
         <v/>
       </c>
       <c r="F4" s="2" t="n">
-        <v>3600</v>
+        <v>6075</v>
       </c>
       <c r="G4" t="n">
         <v>60</v>
@@ -643,17 +643,17 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E6" s="2">
         <f>D6*125</f>
         <v/>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1600</v>
+        <v>750</v>
       </c>
       <c r="G6" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="H6" s="2">
         <f>G6*125</f>
@@ -792,20 +792,20 @@
         <v/>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1600</v>
+        <v>1700</v>
       </c>
       <c r="G9" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H9" s="2">
         <f>G9*125</f>
         <v/>
       </c>
       <c r="I9" s="2" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="J9" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="K9" s="2">
         <f>J9*125</f>
@@ -841,10 +841,10 @@
         <v/>
       </c>
       <c r="F10" s="2" t="n">
-        <v>1300</v>
+        <v>2150</v>
       </c>
       <c r="G10" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="H10" s="2">
         <f>G10*125</f>
@@ -883,14 +883,14 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E11" s="2">
         <f>D11*125</f>
         <v/>
       </c>
       <c r="F11" s="2" t="n">
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
         <v>24</v>
@@ -900,10 +900,10 @@
         <v/>
       </c>
       <c r="I11" s="2" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K11" s="2">
         <f>J11*125</f>
@@ -1123,17 +1123,17 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E16" s="2">
         <f>D16*125</f>
         <v/>
       </c>
       <c r="F16" s="2" t="n">
-        <v>900</v>
+        <v>1700</v>
       </c>
       <c r="G16" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H16" s="2">
         <f>G16*125</f>
@@ -1172,17 +1172,17 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E17" s="2">
         <f>D17*125</f>
         <v/>
       </c>
       <c r="F17" s="2" t="n">
-        <v>1100</v>
+        <v>1700</v>
       </c>
       <c r="G17" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="H17" s="2">
         <f>G17*125</f>
@@ -1221,17 +1221,17 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18" s="2">
         <f>D18*125</f>
         <v/>
       </c>
       <c r="F18" s="2" t="n">
-        <v>300</v>
+        <v>650</v>
       </c>
       <c r="G18" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="H18" s="2">
         <f>G18*125</f>
@@ -1277,20 +1277,20 @@
         <v/>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1450</v>
+        <v>1150</v>
       </c>
       <c r="G19" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H19" s="2">
         <f>G19*125</f>
         <v/>
       </c>
       <c r="I19" s="2" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K19" s="2">
         <f>J19*125</f>
@@ -1671,12 +1671,12 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>FPB-HW-B (300) relocated; 44x20 transfer duct relocated; (2) 12x12 grilles relocated to 5P / 7P Meeting; 12ø branch rerouted.</t>
+          <t>44x20 transfer duct relocated; (2) 12x12 grilles relocated to 5P / 7P Meeting; 12ø branch rerouted.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Disconnect and remove affected duct, fittings and grilles. Relocate FPB-HW-B, install 44x20 transfer duct and 12ø branch at new locations, F&amp;I (2) 12x12 grilles.</t>
+          <t>Disconnect and remove affected duct, fittings and grilles. Install 44x20 transfer duct and 12ø branch at new locations.</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Remove grilles and their duct connections; fabricate and install TD 48x24, F&amp;I 12x12 and 18x12 grilles with duct connections at new locations.</t>
+          <t>Remove grilles and their duct connections; fabricate and install TD 48x24, relocate 12x12 and 18x12 grilles with duct connections at new locations.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Snowflake COP-SF-05 breakdown rev 2: 31st floor area amounts per second markup
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WgFPTBsAevVc5EmsheUHsa
</commit_message>
<xml_diff>
--- a/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
+++ b/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
@@ -1123,7 +1123,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E16" s="2">
         <f>D16*125</f>
@@ -1182,7 +1182,7 @@
         <v>1700</v>
       </c>
       <c r="G17" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H17" s="2">
         <f>G17*125</f>
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E18" s="2">
         <f>D18*125</f>
@@ -1270,14 +1270,14 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E19" s="2">
         <f>D19*125</f>
         <v/>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1150</v>
+        <v>900</v>
       </c>
       <c r="G19" t="n">
         <v>12</v>
@@ -1353,7 +1353,7 @@
       <c r="B21" s="3" t="inlineStr"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>31th floor total</t>
+          <t>31st floor total</t>
         </is>
       </c>
       <c r="D21" s="3">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Remove affected branch fitting; fabricate and install (2) 44x22 lined transfer ducts.</t>
+          <t>Fabricate and install (2) 44x22 lined transfer ducts.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Snowflake COP-SF-05 breakdown rev 3: condensed to 6 pages, 2 per floor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MrzjxMHPNYC7yfRdi1WDkq
</commit_message>
<xml_diff>
--- a/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
+++ b/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Breakdown by area" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Area scope" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Breakdown by area" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Area scope" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Snowflake COP-SF-05 rev 4 (partial): 31st floor per markup, 30th floor text deletions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MrzjxMHPNYC7yfRdi1WDkq
</commit_message>
<xml_diff>
--- a/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
+++ b/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
@@ -459,7 +459,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>COP-SF-05 Bulletin 3 Revision - Snowflake Fitout, 7 Times Square Fl 29-31 - Northern Wolves AC - 09/30/2026</t>
+          <t>COP-SF-05 Bulletin 3 Revision - Snowflake Fitout, 7 Times Square Fl 29-31 - Northern Wolves AC - 10/01/2026</t>
         </is>
       </c>
     </row>
@@ -1021,18 +1021,18 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Zoom rooms, northwest - transfer ducts</t>
+          <t>Zoom rooms, northwest - transfers</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="2">
         <f>D14*125</f>
         <v/>
       </c>
       <c r="F14" s="2" t="n">
-        <v>330</v>
+        <v>530</v>
       </c>
       <c r="G14" t="n">
         <v>6</v>
@@ -1070,11 +1070,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Transfer duct TD 32x16, north</t>
+          <t>Transfer TD 32x16, north</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="2">
         <f>D15*125</f>
@@ -1084,7 +1084,7 @@
         <v>300</v>
       </c>
       <c r="G15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H15" s="2">
         <f>G15*125</f>
@@ -1133,7 +1133,7 @@
         <v>1700</v>
       </c>
       <c r="G16" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H16" s="2">
         <f>G16*125</f>
@@ -1179,10 +1179,10 @@
         <v/>
       </c>
       <c r="F17" s="2" t="n">
-        <v>1700</v>
+        <v>1750</v>
       </c>
       <c r="G17" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H17" s="2">
         <f>G17*125</f>
@@ -1217,11 +1217,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Transfer duct TD 32x16, southwest</t>
+          <t>Transfer TD 32x16, southwest</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E18" s="2">
         <f>D18*125</f>
@@ -1231,7 +1231,7 @@
         <v>650</v>
       </c>
       <c r="G18" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H18" s="2">
         <f>G18*125</f>
@@ -1270,14 +1270,14 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E19" s="2">
         <f>D19*125</f>
         <v/>
       </c>
       <c r="F19" s="2" t="n">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="G19" t="n">
         <v>12</v>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Disconnect and remove 12x10 branch and (2) C(220). Install 10ø branch, 40x20 transfer duct, rework 16x12 branch. F&amp;I G(440) linear diffuser with plenum, relocate G(400) diffusers.</t>
+          <t>Disconnect and remove 12x10 branch and (2) C(220). Install 10ø branch, 40x20 transfer duct, rework 16x12 branch. F&amp;I G(440).</t>
         </is>
       </c>
     </row>
@@ -1666,12 +1666,12 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>FPB-HW-B (300) with supply connections; 44x20 transfer duct; (2) 12x12 grilles; 12ø branch to FPB-HW-D (1200).</t>
+          <t>44x20 transfer duct; (2) 12x12 grilles; 12ø branch to FPB-HW-D (1200).</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>44x20 transfer duct relocated; (2) 12x12 grilles relocated to 5P / 7P Meeting; 12ø branch rerouted.</t>
+          <t>(2) 12x12 grilles relocated to 5P / 7P Meeting; 12ø branch rerouted.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -1691,12 +1691,12 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Zoom rooms, northwest - transfer ducts</t>
+          <t>Zoom rooms, northwest - transfers</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>(1) transfer duct (not sized on Addendum 1).</t>
+          <t>(1) transfer.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Remove existing transfer duct; fabricate and install TD 24x12 and TD 18x12.</t>
+          <t>Mark-up the wall openings, furnish and install (4) transfer grilles.</t>
         </is>
       </c>
     </row>
@@ -1721,22 +1721,22 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Transfer duct TD 32x16, north</t>
+          <t>Transfer TD 32x16, north</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Transfer duct as installed per Addendum 1 (not sized on Addendum 1).</t>
+          <t>Smaller transfer.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Transfer duct revised to TD 32x16.</t>
+          <t>New increased size for wall transfer and (2) grilles.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Remove installed transfer duct; fabricate and install TD 32x16.</t>
+          <t>Mark-up the wall openings, furnish and install (2) transfer grilles.</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>No transfer ducts; volume damper at FPB-HW-B (500) branch.</t>
+          <t>No transfer ducts.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1811,22 +1811,22 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Transfer duct TD 32x16, southwest</t>
+          <t>Transfer TD 32x16, southwest</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Transfer duct and duct elbow as installed per Addendum 1, next to the 12x8 branch.</t>
+          <t>Transfer and duct elbow as installed per Addendum 1, next to the 12x8 branch.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Transfer duct revised to TD 32x16; elbow deleted.</t>
+          <t>Transfer revised to TD 32x16; 12x8 offset shifted to fit transfer.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Remove installed transfer duct and elbow; fabricate and install TD 32x16.</t>
+          <t>Remove installed transfer and elbow; fabricate and install new offset, F/I (2) 32x16 transfer grilles.</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Remove grilles and their duct connections; fabricate and install TD 48x24, relocate 12x12 and 18x12 grilles with duct connections at new locations.</t>
+          <t>Remove grilles and their duct connections; mark-up the wall openings, furnish and install (2) 48x24 transfer grilles; relocate 12x12 and 18x12 grilles with duct connections at new locations.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Snowflake COP-SF-05 rev 4: 29th / 30th per second markup, total back to $66,780
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MrzjxMHPNYC7yfRdi1WDkq
</commit_message>
<xml_diff>
--- a/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
+++ b/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
@@ -552,7 +552,7 @@
         <v/>
       </c>
       <c r="F4" s="2" t="n">
-        <v>6075</v>
+        <v>4875</v>
       </c>
       <c r="G4" t="n">
         <v>60</v>
@@ -594,14 +594,14 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E5" s="2">
         <f>D5*125</f>
         <v/>
       </c>
       <c r="F5" s="2" t="n">
-        <v>3900</v>
+        <v>4975</v>
       </c>
       <c r="G5" t="n">
         <v>50</v>
@@ -650,10 +650,10 @@
         <v/>
       </c>
       <c r="F6" s="2" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
       <c r="G6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H6" s="2">
         <f>G6*125</f>
@@ -785,17 +785,17 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E9" s="2">
         <f>D9*125</f>
         <v/>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1700</v>
+        <v>3800</v>
       </c>
       <c r="G9" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="H9" s="2">
         <f>G9*125</f>
@@ -841,10 +841,10 @@
         <v/>
       </c>
       <c r="F10" s="2" t="n">
-        <v>2150</v>
+        <v>2400</v>
       </c>
       <c r="G10" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="H10" s="2">
         <f>G10*125</f>
@@ -883,17 +883,17 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E11" s="2">
         <f>D11*125</f>
         <v/>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="G11" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="H11" s="2">
         <f>G11*125</f>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>Disconnect and remove installed 46x16 section and branch connections. Fabricate and install 22x10 / 30x10 duct and round branches with insulation, reconnect terminal units.</t>
+          <t>Disconnect and remove installed 46x16 section and branch connections. Fabricate and install 22x10 / 30x10 duct and round branches with insulation.</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Disconnect and remove installed 56x16 main. Fabricate and install 42x12 main with insulation, reconnect branch takeoffs (FPB-HW-E, FPB-B (260)).</t>
+          <t>Disconnect and remove installed 56x16 main. Fabricate and install 42x12 main with insulation.</t>
         </is>
       </c>
     </row>
@@ -1611,12 +1611,12 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>12x10 branch and (2) C(220) deleted, replaced with 10ø branch to (1) new G(440) linear diffuser. New 40x20 transfer duct at F&amp;B Storage 30.14. G(400) linear diffusers relocated along the 16x12 branch.</t>
+          <t>12x10 branch and (2) C(220) deleted, replaced with 10ø branch to (1) new G(440) linear diffuser. New 40x20 transfer duct at F&amp;B Storage 30.14. G(400) diffusers relocated along the 16x12 branch.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Disconnect and remove 12x10 branch and (2) C(220). Install 10ø branch, 40x20 transfer duct, rework 16x12 branch. F&amp;I G(440).</t>
+          <t>Disconnect and remove 12x10 branch and (2) C(220). Install 10ø branch, 40x20 transfer duct, rework 16x12 branch. F&amp;I G(440). F/I (2) 40x20 wall transfer grilles.</t>
         </is>
       </c>
     </row>
@@ -1641,12 +1641,12 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>(2) new 48x24 transfer ducts.</t>
+          <t>(2) new 48x24 transfer ducts with 1" AL.</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Fabricate and install (2) 48x24 lined transfer ducts.</t>
+          <t>Fabricate and install (2) 48x24 lined transfer ducts and (2) 48x24 transfer return grilles.</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Disconnect and remove affected duct, fittings and grilles. Install 44x20 transfer duct and 12ø branch at new locations.</t>
+          <t>Disconnect and remove affected duct, FSD, fittings. Install 44x20 duct, FSD with angles, and 12ø branch at new locations.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Snowflake COP-SF-05 rev 5: area 29-2 excluded, revised total $53,555
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MrzjxMHPNYC7yfRdi1WDkq
</commit_message>
<xml_diff>
--- a/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
+++ b/Reference/Change Orders/2026-09 Snowflake COP-SF-05 Bulletin 3/COP-SF-05 Bulletin 3 - Detailed Breakdown.xlsx
@@ -585,26 +585,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>29-2</t>
+          <t>29-3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Supply main resized 56x16 to 42x12</t>
+          <t>FPB-HW-E (1400) relocation and discharge reroute</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E5" s="2">
         <f>D5*125</f>
         <v/>
       </c>
       <c r="F5" s="2" t="n">
-        <v>4975</v>
+        <v>500</v>
       </c>
       <c r="G5" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="H5" s="2">
         <f>G5*125</f>
@@ -634,30 +634,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>29-3</t>
+          <t>29-2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>FPB-HW-E (1400) relocation and discharge reroute</t>
+          <t>Supply main resized 56x16 to 42x12 - Excluded - per Bulletin 3 the existing 56x16 main on the 29th floor remains as installed; no change to this ductwork.</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" s="2">
-        <f>D6*125</f>
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>6</v>
-      </c>
-      <c r="H6" s="2">
-        <f>G6*125</f>
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>0</v>
@@ -665,16 +663,14 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="2">
-        <f>J6*125</f>
-        <v/>
+      <c r="K6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="L6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M6" s="2">
-        <f>E6+F6+H6+I6+K6+L6</f>
-        <v/>
+      <c r="M6" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1402,7 +1398,7 @@
       <c r="B22" s="3" t="inlineStr"/>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>TOTAL COP-SF-05</t>
+          <t>TOTAL COP-SF-05 (revised)</t>
         </is>
       </c>
       <c r="D22" s="3">
@@ -1457,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1533,7 +1529,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>29-2</t>
+          <t>29-3</t>
         </is>
       </c>
       <c r="B3" s="6" t="n">
@@ -1541,59 +1537,59 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Supply main resized 56x16 to 42x12</t>
+          <t>FPB-HW-E (1400) relocation and discharge reroute</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>56x16 supply main, approx. 44 LF, top el. 11'-1" / bottom el. 9'-9", Break Rm 29.57 to P.E.</t>
+          <t>FPB-HW-E (1400) with inlet and 30x10 discharge to the G(400) / G(200) linear diffusers along the northeast wall.</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Main resized to 42x12 on the same route, top el. 11'-1" / bottom el. 10'-1".</t>
+          <t>FPB-HW-E relocated; inlet connection and 30x10 discharge elbow rerouted.</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Disconnect and remove installed 56x16 main. Fabricate and install 42x12 main with insulation.</t>
+          <t>Disconnect inlet and discharge, relocate and rehang FPB-HW-E, fabricate and install new inlet and 30x10 discharge fittings, reconnect.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>29-3</t>
+          <t>30-1</t>
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>FPB-HW-E (1400) relocation and discharge reroute</t>
+          <t>IT Build Rm 30.23 / F&amp;B Storage 30.14 / west dining</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>FPB-HW-E (1400) with inlet and 30x10 discharge to the G(400) / G(200) linear diffusers along the northeast wall.</t>
+          <t>12x10 branch with (2) C(220) ceiling diffusers; G(400) linear diffuser run on 16x12 branch.</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>FPB-HW-E relocated; inlet connection and 30x10 discharge elbow rerouted.</t>
+          <t>12x10 branch and (2) C(220) deleted, replaced with 10ø branch to (1) new G(440) linear diffuser. New 40x20 transfer duct at F&amp;B Storage 30.14. G(400) diffusers relocated along the 16x12 branch.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Disconnect inlet and discharge, relocate and rehang FPB-HW-E, fabricate and install new inlet and 30x10 discharge fittings, reconnect.</t>
+          <t>Disconnect and remove 12x10 branch and (2) C(220). Install 10ø branch, 40x20 transfer duct, rework 16x12 branch. F&amp;I G(440). F/I (2) 40x20 wall transfer grilles.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>30-1</t>
+          <t>30-2</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">
@@ -1601,29 +1597,29 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>IT Build Rm 30.23 / F&amp;B Storage 30.14 / west dining</t>
+          <t>Lounge 30.02 - new transfer ducts</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>12x10 branch with (2) C(220) ceiling diffusers; G(400) linear diffuser run on 16x12 branch.</t>
+          <t>No transfer ducts at Lounge 30.02 walls.</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>12x10 branch and (2) C(220) deleted, replaced with 10ø branch to (1) new G(440) linear diffuser. New 40x20 transfer duct at F&amp;B Storage 30.14. G(400) diffusers relocated along the 16x12 branch.</t>
+          <t>(2) new 48x24 transfer ducts with 1" AL.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Disconnect and remove 12x10 branch and (2) C(220). Install 10ø branch, 40x20 transfer duct, rework 16x12 branch. F&amp;I G(440). F/I (2) 40x20 wall transfer grilles.</t>
+          <t>Fabricate and install (2) 48x24 lined transfer ducts and (2) 48x24 transfer return grilles.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>30-2</t>
+          <t>30-3</t>
         </is>
       </c>
       <c r="B6" s="6" t="n">
@@ -1631,59 +1627,59 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Lounge 30.02 - new transfer ducts</t>
+          <t>Meeting Rms 30.04 / 30.05, Storage 30.09, Vestibule 30.07</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>No transfer ducts at Lounge 30.02 walls.</t>
+          <t>44x20 transfer duct; (2) 12x12 grilles; 12ø branch to FPB-HW-D (1200).</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>(2) new 48x24 transfer ducts with 1" AL.</t>
+          <t>(2) 12x12 grilles relocated to 5P / 7P Meeting; 12ø branch rerouted.</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Fabricate and install (2) 48x24 lined transfer ducts and (2) 48x24 transfer return grilles.</t>
+          <t>Disconnect and remove affected duct, FSD, fittings. Install 44x20 duct, FSD with angles, and 12ø branch at new locations.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>30-3</t>
+          <t>31-1</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Meeting Rms 30.04 / 30.05, Storage 30.09, Vestibule 30.07</t>
+          <t>Zoom rooms, northwest - transfers</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>44x20 transfer duct; (2) 12x12 grilles; 12ø branch to FPB-HW-D (1200).</t>
+          <t>(1) transfer.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>(2) 12x12 grilles relocated to 5P / 7P Meeting; 12ø branch rerouted.</t>
+          <t>TD 24x12 and new TD 18x12.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Disconnect and remove affected duct, FSD, fittings. Install 44x20 duct, FSD with angles, and 12ø branch at new locations.</t>
+          <t>Mark-up the wall openings, furnish and install (4) transfer grilles.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>31-1</t>
+          <t>31-2</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
@@ -1691,29 +1687,29 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Zoom rooms, northwest - transfers</t>
+          <t>Transfer TD 32x16, north</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>(1) transfer.</t>
+          <t>Smaller transfer.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>TD 24x12 and new TD 18x12.</t>
+          <t>New increased size for wall transfer and (2) grilles.</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Mark-up the wall openings, furnish and install (4) transfer grilles.</t>
+          <t>Mark-up the wall openings, furnish and install (2) transfer grilles.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>31-2</t>
+          <t>31-3</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
@@ -1721,29 +1717,29 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Transfer TD 32x16, north</t>
+          <t>Storage 31.02 - new transfer ducts</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Smaller transfer.</t>
+          <t>No transfer ducts.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>New increased size for wall transfer and (2) grilles.</t>
+          <t>(2) new 44x22 transfer ducts.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Mark-up the wall openings, furnish and install (2) transfer grilles.</t>
+          <t>Fabricate and install (2) 44x22 lined transfer ducts.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>31-3</t>
+          <t>31-4</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
@@ -1751,29 +1747,29 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Storage 31.02 - new transfer ducts</t>
+          <t>Coffee Bar 31.12 - transfer ducts and main fitting</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>No transfer ducts.</t>
+          <t>36x18 main with elbow at Coffee Bar 31.12; no transfer ducts.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>(2) new 44x22 transfer ducts.</t>
+          <t>(2) new TD 28x16; 36x18 main elbow reconfigured.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Fabricate and install (2) 44x22 lined transfer ducts.</t>
+          <t>Disconnect and remove 36x18 elbow; fabricate and install new fitting and (2) TD 28x16.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>31-4</t>
+          <t>31-5</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
@@ -1781,29 +1777,29 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Coffee Bar 31.12 - transfer ducts and main fitting</t>
+          <t>Transfer TD 32x16, southwest</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>36x18 main with elbow at Coffee Bar 31.12; no transfer ducts.</t>
+          <t>Transfer and duct elbow as installed per Addendum 1, next to the 12x8 branch.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>(2) new TD 28x16; 36x18 main elbow reconfigured.</t>
+          <t>Transfer revised to TD 32x16; 12x8 offset shifted to fit transfer.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Disconnect and remove 36x18 elbow; fabricate and install new fitting and (2) TD 28x16.</t>
+          <t>Remove installed transfer and elbow; fabricate and install new offset, F/I (2) 32x16 transfer grilles.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>31-5</t>
+          <t>31-6</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
@@ -1811,50 +1807,20 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Transfer TD 32x16, southwest</t>
+          <t>Storage 31.15 / Room 31.16, southeast</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Transfer and duct elbow as installed per Addendum 1, next to the 12x8 branch.</t>
+          <t>12x12 and 18x12 grilles at previous locations; no transfer duct at Storage 31.15.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Transfer revised to TD 32x16; 12x8 offset shifted to fit transfer.</t>
+          <t>New TD 48x24; 12x12 and 18x12 grilles relocated.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Remove installed transfer and elbow; fabricate and install new offset, F/I (2) 32x16 transfer grilles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>31-6</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Storage 31.15 / Room 31.16, southeast</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>12x12 and 18x12 grilles at previous locations; no transfer duct at Storage 31.15.</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>New TD 48x24; 12x12 and 18x12 grilles relocated.</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Remove grilles and their duct connections; mark-up the wall openings, furnish and install (2) 48x24 transfer grilles; relocate 12x12 and 18x12 grilles with duct connections at new locations.</t>
         </is>

</xml_diff>